<commit_message>
feat: support Bank Norwegian "Reservert" (pending) transactions
Pending transactions have no date fields. Keep them visible in the
transaction list but exclude them from the monthly heatmap and sums.
Detection is by Type === "Reservert" only.

- Date fields on RawTransaction/Transaction are now nullable
- Parser normalizes missing dates to null
- App.tsx period filter and initial-range calc skip null dates
- statistics.ts filters out undated rows before d3.rollup
- Fixture adds one Reservert row; tests cover parser, statistics, E2E
- Design doc at docs/reservert-pending-transactions.md
</commit_message>
<xml_diff>
--- a/v2/e2e/fixtures/test-transactions-bank-norwegian.xlsx
+++ b/v2/e2e/fixtures/test-transactions-bank-norwegian.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="32">
   <si>
     <t>TransactionDate</t>
   </si>
@@ -98,6 +98,15 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Pending at ZARA</t>
+  </si>
+  <si>
+    <t>Reservert</t>
+  </si>
+  <si>
+    <t>Clothing Stores, MEN, WOMEN, and CHIL</t>
   </si>
 </sst>
 </file>
@@ -474,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -685,6 +694,32 @@
       </c>
       <c r="K6" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7">
+        <v>-299</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7">
+        <v>-299</v>
+      </c>
+      <c r="J7" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>